<commit_message>
Update Website Logics spreadsheet
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Website Logics.xlsx
+++ b/Website Logics.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\veejs\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\veejs\Viscraft\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{53A1F5E3-8821-49D6-8C3C-44DE2E6FF13D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0D57259-8049-413A-B1D8-E9B3108348B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{B52DBFA1-18E2-4400-B0CB-17862293058C}"/>
   </bookViews>
@@ -275,13 +275,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -613,13 +612,13 @@
       <c r="A1" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
     </row>
@@ -1300,7 +1299,7 @@
         <v>34</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="C50" s="1" t="s">
         <v>61</v>

</xml_diff>